<commit_message>
add brand assumptions, energy benchmarks and electricity tariffs
</commit_message>
<xml_diff>
--- a/ghg_inventory_2025.xlsx
+++ b/ghg_inventory_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kirstyshearer/Desktop/job-search/projects/fashion-brand-carbon-footprint/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED340C30-1994-9C44-B82B-7A86887C01B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_D13AD20C306C3E6144E30106F3CC02954FE05B8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1020" yWindow="680" windowWidth="14200" windowHeight="18460" activeTab="4" xr2:uid="{1B2B80B6-3D3F-1D4E-AD75-2AFF293AF52F}"/>
+    <workbookView xWindow="1040" yWindow="660" windowWidth="14200" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -19,11 +19,8 @@
     <sheet name="Calculations" sheetId="4" r:id="rId4"/>
     <sheet name="Summary" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -35,22 +32,229 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="65">
+  <si>
+    <t>Section</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Value</t>
+  </si>
+  <si>
+    <t>Unit</t>
+  </si>
+  <si>
+    <t>Source / reasoning</t>
+  </si>
+  <si>
+    <t>Staff</t>
+  </si>
+  <si>
+    <t>Shop staff</t>
+  </si>
+  <si>
+    <t>people</t>
+  </si>
+  <si>
+    <t>Small shop staffed on a rota</t>
+  </si>
+  <si>
+    <t>Studio staff</t>
+  </si>
+  <si>
+    <t>Design, production, sourcing and online orders</t>
+  </si>
+  <si>
+    <t>Total staff</t>
+  </si>
+  <si>
+    <t>Formula</t>
+  </si>
+  <si>
+    <t>Buildings</t>
+  </si>
+  <si>
+    <t>Shop floor area</t>
+  </si>
+  <si>
+    <t>m²</t>
+  </si>
+  <si>
+    <t>Based on independent designer shops in London</t>
+  </si>
+  <si>
+    <t>Desk space per person</t>
+  </si>
+  <si>
+    <t>m² per person</t>
+  </si>
+  <si>
+    <t>https://www.bco.org.uk/bco-announces-new-recommendations-for-greener-and-healthier-offices</t>
+  </si>
+  <si>
+    <t>Studio workroom area</t>
+  </si>
+  <si>
+    <t>Pattern cutting, sampling, fabric storage, fittings</t>
+  </si>
+  <si>
+    <t>Studio floor area</t>
+  </si>
+  <si>
+    <t>Formula: studio staff × desk space + workroom</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Shop electricity benchmark</t>
+  </si>
+  <si>
+    <t>kWh per m² per year</t>
+  </si>
+  <si>
+    <t>ND-NEED 2026 edition (published Sept 2026), Table 9A, Shops, 2024 median for England and Wales</t>
+  </si>
+  <si>
+    <t>Shop gas benchmark</t>
+  </si>
+  <si>
+    <t>ND-NEED 2026 edition (published Sept 2026), Table 9C, Shops, 2024 median for England and Wales</t>
+  </si>
+  <si>
+    <t>Studio electricity benchmark</t>
+  </si>
+  <si>
+    <t>ND-NEED 2026 edition (published Sept 2026), Table 9A, Offices, 2024 median for England and Wales. Offices used for the whole studio, so this probably underestimates electricity for the workroom machines (sewing machines, irons, steamers).</t>
+  </si>
+  <si>
+    <t>Studio gas benchmark</t>
+  </si>
+  <si>
+    <t>ND-NEED 2026 edition (published Sept 2026), Table 9C, Offices, 2024 median for England and Wales.</t>
+  </si>
+  <si>
+    <t>Shop electricity use</t>
+  </si>
+  <si>
+    <t>kWh per year</t>
+  </si>
+  <si>
+    <t>Formula: floor area × benchmark</t>
+  </si>
+  <si>
+    <t>Shop gas use</t>
+  </si>
+  <si>
+    <t>Studio electricity use</t>
+  </si>
+  <si>
+    <t>Studio gas use</t>
+  </si>
+  <si>
+    <t>Shop electricity tariff</t>
+  </si>
+  <si>
+    <t>Landlord-supplied, tariff unknown</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>Leased retail unit: landlord buys the electricity and recharges it in the service charge. Decides the market-based Scope 2 factor.</t>
+  </si>
+  <si>
+    <t>Studio electricity tariff</t>
+  </si>
+  <si>
+    <t>100% renewable, backed by REGOs</t>
+  </si>
+  <si>
+    <t>Brand's own contract, chosen by the brand. Decides the market-based Scope 2 factor.</t>
+  </si>
+  <si>
+    <t>Scope 3 (later)</t>
+  </si>
+  <si>
+    <t>Garments made per year</t>
+  </si>
+  <si>
+    <t>garments</t>
+  </si>
+  <si>
+    <t>Share made in the UK</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Online orders per year</t>
+  </si>
+  <si>
+    <t>orders</t>
+  </si>
+  <si>
+    <t>Business trips per year</t>
+  </si>
+  <si>
+    <t>trips</t>
+  </si>
+  <si>
+    <t>Brand name</t>
+  </si>
+  <si>
+    <t>Reporting period</t>
+  </si>
+  <si>
+    <t>1 January to 31 December 2025</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>GHG Protocol Corporate Standard</t>
+  </si>
+  <si>
+    <t>Emission factors</t>
+  </si>
+  <si>
+    <t>DESNZ conversion factors 2025, condensed set</t>
+  </si>
+  <si>
+    <t>Colour key</t>
+  </si>
+  <si>
+    <t>Blue text = typed input. Black text = formula.</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
     </font>
   </fonts>
   <fills count="2">
@@ -73,8 +277,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -408,45 +614,457 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A6BCAE7-0E53-AB4D-ADE2-409051DF38CC}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="7" max="7" width="31.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{490F8E6C-4514-6449-8D2A-5B939C0919E6}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="70" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="2">
+        <v>9</v>
+      </c>
+      <c r="D3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <f>C2+C3</f>
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2">
+        <v>130</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="2">
+        <v>70</v>
+      </c>
+      <c r="D7" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8">
+        <f>C3*C6+C7</f>
+        <v>160</v>
+      </c>
+      <c r="D8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" s="2">
+        <v>108.01</v>
+      </c>
+      <c r="D9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C10" s="2">
+        <v>190.08</v>
+      </c>
+      <c r="D10" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="2">
+        <v>62.8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="E11" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="2">
+        <v>147.54</v>
+      </c>
+      <c r="D12" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13">
+        <f>C5*C9</f>
+        <v>14041.300000000001</v>
+      </c>
+      <c r="D13" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14">
+        <f>C5*C10</f>
+        <v>24710.400000000001</v>
+      </c>
+      <c r="D14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E14" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15">
+        <f>C8*C11</f>
+        <v>10048</v>
+      </c>
+      <c r="D15" t="s">
+        <v>35</v>
+      </c>
+      <c r="E15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C16">
+        <f>C8*C12</f>
+        <v>23606.399999999998</v>
+      </c>
+      <c r="D16" t="s">
+        <v>35</v>
+      </c>
+      <c r="E16" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" t="s">
+        <v>48</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" t="s">
+        <v>55</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{005A3E7A-F27C-8747-8173-BE5887F53A1A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAE93EDF-5C36-7746-870B-C28DAADDAA4C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44D2F417-B508-254E-8384-A99133E72FC9}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
add natural gas and UK electricity factors
</commit_message>
<xml_diff>
--- a/ghg_inventory_2025.xlsx
+++ b/ghg_inventory_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kirstyshearer/Desktop/job-search/projects/fashion-brand-carbon-footprint/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_D13AD20C306C3E6144E30106F3CC02954FE05B8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C5C5327-025B-8F41-BD92-479FBCBD6540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="660" windowWidth="14200" windowHeight="18460" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1040" yWindow="660" windowWidth="14200" windowHeight="18460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="89">
   <si>
     <t>Section</t>
   </si>
@@ -222,6 +222,12 @@
     <t>GHG Protocol Corporate Standard</t>
   </si>
   <si>
+    <t>Boundary</t>
+  </si>
+  <si>
+    <t>Operational control</t>
+  </si>
+  <si>
     <t>Emission factors</t>
   </si>
   <si>
@@ -232,13 +238,79 @@
   </si>
   <si>
     <t>Blue text = typed input. Black text = formula.</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Factor</t>
+  </si>
+  <si>
+    <t>Scope</t>
+  </si>
+  <si>
+    <t>Source (DESNZ sheet, row label, year and set)</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>GAS_NAT</t>
+  </si>
+  <si>
+    <t>Natural gas</t>
+  </si>
+  <si>
+    <t>Scope 1</t>
+  </si>
+  <si>
+    <t>ELEC_UK_LOC</t>
+  </si>
+  <si>
+    <t>UK grid electricity, location-based</t>
+  </si>
+  <si>
+    <t>Scope 2</t>
+  </si>
+  <si>
+    <t>ELEC_SHOP_MKT</t>
+  </si>
+  <si>
+    <t>Shop electricity, market-based</t>
+  </si>
+  <si>
+    <t>ELEC_STUDIO_MKT</t>
+  </si>
+  <si>
+    <t>Studio electricity, market-based</t>
+  </si>
+  <si>
+    <t>kg CO2e per kWh (Gross CV)</t>
+  </si>
+  <si>
+    <t>DESNZ 2025 condensed set, Fuels sheet, Natural gas, kWh (Gross CV), kg CO2e column</t>
+  </si>
+  <si>
+    <t>Gross CV to match the activity data. ND-NEED kWh comes from metered supplier data, which, like UK gas bills, is on a gross basis.</t>
+  </si>
+  <si>
+    <t>DESNZ 2025 condensed set, UK Electricity sheet, Electricity generated, kWh, kg CO2e column</t>
+  </si>
+  <si>
+    <t>kg CO2e per kWh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generation factor used for Scope 2, as DESNZ advises - it covers emissions from producing the electricity the brand buys. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -249,6 +321,11 @@
     <font>
       <b/>
       <sz val="12"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0000FF"/>
       <name val="Aptos Narrow"/>
     </font>
     <font>
@@ -277,10 +354,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -615,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -659,6 +737,14 @@
       </c>
       <c r="B5" t="s">
         <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" t="s">
+        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -1045,9 +1131,117 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="36" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="7" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C2" s="3">
+        <v>0.18296000000000001</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
add market-based factors and residual mix calculation
</commit_message>
<xml_diff>
--- a/ghg_inventory_2025.xlsx
+++ b/ghg_inventory_2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kirstyshearer/Desktop/job-search/projects/fashion-brand-carbon-footprint/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C5C5327-025B-8F41-BD92-479FBCBD6540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6801B652-3D7B-7841-AF8F-348B5E4C5E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1040" yWindow="660" windowWidth="14200" windowHeight="18460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,8 +16,9 @@
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="Assumptions" sheetId="2" r:id="rId2"/>
     <sheet name="Emission factors" sheetId="3" r:id="rId3"/>
-    <sheet name="Calculations" sheetId="4" r:id="rId4"/>
-    <sheet name="Summary" sheetId="5" r:id="rId5"/>
+    <sheet name="Residual mix" sheetId="6" r:id="rId4"/>
+    <sheet name="Calculations" sheetId="4" r:id="rId5"/>
+    <sheet name="Summary" sheetId="5" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="104">
   <si>
     <t>Section</t>
   </si>
@@ -304,13 +305,61 @@
   </si>
   <si>
     <t xml:space="preserve">Generation factor used for Scope 2, as DESNZ advises - it covers emissions from producing the electricity the brand buys. </t>
+  </si>
+  <si>
+    <t>0 as REGO-backed renewable.</t>
+  </si>
+  <si>
+    <t>GHG Protocol Scope 2 Guidance (market-based method, Scope 2 Quality Criteria).</t>
+  </si>
+  <si>
+    <t>Coal</t>
+  </si>
+  <si>
+    <t>Natural Gas</t>
+  </si>
+  <si>
+    <t>Nuclear</t>
+  </si>
+  <si>
+    <t>Renewables</t>
+  </si>
+  <si>
+    <t>Other Fuels</t>
+  </si>
+  <si>
+    <t>Energy Source (%)</t>
+  </si>
+  <si>
+    <t>Intensity (g/kWh)</t>
+  </si>
+  <si>
+    <t>Weighted Average</t>
+  </si>
+  <si>
+    <t>Contribution (g/kWh)</t>
+  </si>
+  <si>
+    <t>Contribution (kg/kWh)</t>
+  </si>
+  <si>
+    <t>kg CO2 per kWh</t>
+  </si>
+  <si>
+    <t>Residual mix used because the landlord's tariff is unknown (emission factor hierarchy). In reality the brand would ask the landlord. Coal - 2024 intensity, since there was no coal generation in 2025</t>
+  </si>
+  <si>
+    <t>Calculated from DESNZ Fuel Mix Disclosure data table, residual fuel mix for April 2025 to March 2026, CO2 intensities for 2025</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="7">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -331,6 +380,24 @@
     <font>
       <sz val="12"/>
       <color rgb="FF0000FF"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0432FF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
@@ -354,17 +421,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FF0432FF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1218,13 +1295,22 @@
       <c r="B4" t="s">
         <v>80</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="C4" s="8">
+        <f>'Residual mix'!E7</f>
+        <v>0.39566500000000004</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>101</v>
+      </c>
       <c r="E4" t="s">
         <v>78</v>
       </c>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="F4" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
@@ -1233,13 +1319,21 @@
       <c r="B5" t="s">
         <v>82</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
+      <c r="C5" s="3">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>87</v>
+      </c>
       <c r="E5" t="s">
         <v>78</v>
       </c>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="F5" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1247,6 +1341,150 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87414153-6F28-2944-A156-CC2E49189BDE}">
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="2" max="2" width="15" style="4" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="18.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="B1" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" t="s">
+        <v>99</v>
+      </c>
+      <c r="E1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B2" s="5">
+        <v>0.114</v>
+      </c>
+      <c r="C2" s="6">
+        <v>921</v>
+      </c>
+      <c r="D2">
+        <f>B2*C2</f>
+        <v>104.994</v>
+      </c>
+      <c r="E2">
+        <f>D2/1000</f>
+        <v>0.104994</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B3" s="5">
+        <v>0.65300000000000002</v>
+      </c>
+      <c r="C3" s="6">
+        <v>365</v>
+      </c>
+      <c r="D3">
+        <f t="shared" ref="D3:D6" si="0">B3*C3</f>
+        <v>238.345</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E7" si="1">D3/1000</f>
+        <v>0.238345</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B4" s="5">
+        <v>7.0999999999999994E-2</v>
+      </c>
+      <c r="C4" s="6">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" s="5">
+        <v>0.108</v>
+      </c>
+      <c r="C5" s="6">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B6" s="5">
+        <v>5.3999999999999999E-2</v>
+      </c>
+      <c r="C6" s="6">
+        <v>969</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>52.326000000000001</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>5.2325999999999998E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>98</v>
+      </c>
+      <c r="D7">
+        <f>SUM(D2:D6)</f>
+        <v>395.66500000000002</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>0.39566500000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="7"/>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="7"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -1255,7 +1493,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>

</xml_diff>

<commit_message>
calculations and summary of Scope 1 and 2 emissions
</commit_message>
<xml_diff>
--- a/ghg_inventory_2025.xlsx
+++ b/ghg_inventory_2025.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kirstyshearer/Desktop/job-search/projects/fashion-brand-carbon-footprint/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6801B652-3D7B-7841-AF8F-348B5E4C5E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A036935-34BA-1646-9313-62B74444CE1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1040" yWindow="660" windowWidth="14200" windowHeight="18460" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1040" yWindow="660" windowWidth="14200" windowHeight="18460" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
-    <sheet name="Assumptions" sheetId="2" r:id="rId2"/>
-    <sheet name="Emission factors" sheetId="3" r:id="rId3"/>
-    <sheet name="Residual mix" sheetId="6" r:id="rId4"/>
-    <sheet name="Calculations" sheetId="4" r:id="rId5"/>
-    <sheet name="Summary" sheetId="5" r:id="rId6"/>
+    <sheet name="Summary" sheetId="5" r:id="rId2"/>
+    <sheet name="Assumptions" sheetId="2" r:id="rId3"/>
+    <sheet name="Emission factors" sheetId="3" r:id="rId4"/>
+    <sheet name="Residual mix" sheetId="6" r:id="rId5"/>
+    <sheet name="Calculations" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="115">
   <si>
     <t>Section</t>
   </si>
@@ -97,9 +97,6 @@
     <t>m² per person</t>
   </si>
   <si>
-    <t>https://www.bco.org.uk/bco-announces-new-recommendations-for-greener-and-healthier-offices</t>
-  </si>
-  <si>
     <t>Studio workroom area</t>
   </si>
   <si>
@@ -181,175 +178,211 @@
     <t>Brand's own contract, chosen by the brand. Decides the market-based Scope 2 factor.</t>
   </si>
   <si>
-    <t>Scope 3 (later)</t>
-  </si>
-  <si>
-    <t>Garments made per year</t>
-  </si>
-  <si>
-    <t>garments</t>
-  </si>
-  <si>
-    <t>Share made in the UK</t>
-  </si>
-  <si>
-    <t>%</t>
-  </si>
-  <si>
-    <t>Online orders per year</t>
-  </si>
-  <si>
-    <t>orders</t>
-  </si>
-  <si>
-    <t>Business trips per year</t>
-  </si>
-  <si>
-    <t>trips</t>
+    <t>Reporting period</t>
+  </si>
+  <si>
+    <t>1 January to 31 December 2025</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>GHG Protocol Corporate Standard</t>
+  </si>
+  <si>
+    <t>Boundary</t>
+  </si>
+  <si>
+    <t>Operational control</t>
+  </si>
+  <si>
+    <t>Emission factors</t>
+  </si>
+  <si>
+    <t>DESNZ conversion factors 2025, condensed set</t>
+  </si>
+  <si>
+    <t>Colour key</t>
+  </si>
+  <si>
+    <t>Blue text = typed input. Black text = formula.</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Factor</t>
+  </si>
+  <si>
+    <t>Scope</t>
+  </si>
+  <si>
+    <t>Source (DESNZ sheet, row label, year and set)</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>GAS_NAT</t>
+  </si>
+  <si>
+    <t>Natural gas</t>
+  </si>
+  <si>
+    <t>Scope 1</t>
+  </si>
+  <si>
+    <t>ELEC_UK_LOC</t>
+  </si>
+  <si>
+    <t>UK grid electricity, location-based</t>
+  </si>
+  <si>
+    <t>Scope 2</t>
+  </si>
+  <si>
+    <t>ELEC_SHOP_MKT</t>
+  </si>
+  <si>
+    <t>Shop electricity, market-based</t>
+  </si>
+  <si>
+    <t>ELEC_STUDIO_MKT</t>
+  </si>
+  <si>
+    <t>Studio electricity, market-based</t>
+  </si>
+  <si>
+    <t>kg CO2e per kWh (Gross CV)</t>
+  </si>
+  <si>
+    <t>DESNZ 2025 condensed set, Fuels sheet, Natural gas, kWh (Gross CV), kg CO2e column</t>
+  </si>
+  <si>
+    <t>Gross CV to match the activity data. ND-NEED kWh comes from metered supplier data, which, like UK gas bills, is on a gross basis.</t>
+  </si>
+  <si>
+    <t>DESNZ 2025 condensed set, UK Electricity sheet, Electricity generated, kWh, kg CO2e column</t>
+  </si>
+  <si>
+    <t>kg CO2e per kWh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generation factor used for Scope 2, as DESNZ advises - it covers emissions from producing the electricity the brand buys. </t>
+  </si>
+  <si>
+    <t>0 as REGO-backed renewable.</t>
+  </si>
+  <si>
+    <t>GHG Protocol Scope 2 Guidance (market-based method, Scope 2 Quality Criteria).</t>
+  </si>
+  <si>
+    <t>Coal</t>
+  </si>
+  <si>
+    <t>Nuclear</t>
+  </si>
+  <si>
+    <t>Renewables</t>
+  </si>
+  <si>
+    <t>Intensity (g/kWh)</t>
+  </si>
+  <si>
+    <t>Contribution (g/kWh)</t>
+  </si>
+  <si>
+    <t>Contribution (kg/kWh)</t>
+  </si>
+  <si>
+    <t>kg CO2 per kWh</t>
+  </si>
+  <si>
+    <t>Residual mix used because the landlord's tariff is unknown (emission factor hierarchy). In reality the brand would ask the landlord. Coal - 2024 intensity, since there was no coal generation in 2025</t>
+  </si>
+  <si>
+    <t>Calculated from DESNZ Fuel Mix Disclosure data table, residual fuel mix for April 2025 to March 2026, CO2 intensities for 2025</t>
+  </si>
+  <si>
+    <t>Shop</t>
+  </si>
+  <si>
+    <t>Studio</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>Location-based</t>
+  </si>
+  <si>
+    <t>Market-based</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Gas</t>
+  </si>
+  <si>
+    <t>Electricity</t>
+  </si>
+  <si>
+    <t>Activity data (kWh)</t>
+  </si>
+  <si>
+    <t>Factor ID</t>
+  </si>
+  <si>
+    <t>Factor unit</t>
+  </si>
+  <si>
+    <t>Emissions (kg CO2e)</t>
+  </si>
+  <si>
+    <t>Emissions (t CO2e)</t>
+  </si>
+  <si>
+    <t>Total emissions (t CO2e)</t>
+  </si>
+  <si>
+    <t>Note:</t>
+  </si>
+  <si>
+    <t>Shop market-based figure is CO2 only (residual mix source)</t>
+  </si>
+  <si>
+    <t>Total (Scope 1+2)</t>
+  </si>
+  <si>
+    <t>Fictional brand</t>
+  </si>
+  <si>
+    <t>Fuel</t>
+  </si>
+  <si>
+    <t>Other fuels</t>
+  </si>
+  <si>
+    <t>Weighted average</t>
+  </si>
+  <si>
+    <t>BCO recommendations on office space per person - https://www.bco.org.uk/bco-announces-new-recommendations-for-greener-and-healthier-offices</t>
   </si>
   <si>
     <t>Brand name</t>
   </si>
   <si>
-    <t>Reporting period</t>
-  </si>
-  <si>
-    <t>1 January to 31 December 2025</t>
-  </si>
-  <si>
-    <t>Standard</t>
-  </si>
-  <si>
-    <t>GHG Protocol Corporate Standard</t>
-  </si>
-  <si>
-    <t>Boundary</t>
-  </si>
-  <si>
-    <t>Operational control</t>
-  </si>
-  <si>
-    <t>Emission factors</t>
-  </si>
-  <si>
-    <t>DESNZ conversion factors 2025, condensed set</t>
-  </si>
-  <si>
-    <t>Colour key</t>
-  </si>
-  <si>
-    <t>Blue text = typed input. Black text = formula.</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>Factor</t>
-  </si>
-  <si>
-    <t>Scope</t>
-  </si>
-  <si>
-    <t>Source (DESNZ sheet, row label, year and set)</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>GAS_NAT</t>
-  </si>
-  <si>
-    <t>Natural gas</t>
-  </si>
-  <si>
-    <t>Scope 1</t>
-  </si>
-  <si>
-    <t>ELEC_UK_LOC</t>
-  </si>
-  <si>
-    <t>UK grid electricity, location-based</t>
-  </si>
-  <si>
-    <t>Scope 2</t>
-  </si>
-  <si>
-    <t>ELEC_SHOP_MKT</t>
-  </si>
-  <si>
-    <t>Shop electricity, market-based</t>
-  </si>
-  <si>
-    <t>ELEC_STUDIO_MKT</t>
-  </si>
-  <si>
-    <t>Studio electricity, market-based</t>
-  </si>
-  <si>
-    <t>kg CO2e per kWh (Gross CV)</t>
-  </si>
-  <si>
-    <t>DESNZ 2025 condensed set, Fuels sheet, Natural gas, kWh (Gross CV), kg CO2e column</t>
-  </si>
-  <si>
-    <t>Gross CV to match the activity data. ND-NEED kWh comes from metered supplier data, which, like UK gas bills, is on a gross basis.</t>
-  </si>
-  <si>
-    <t>DESNZ 2025 condensed set, UK Electricity sheet, Electricity generated, kWh, kg CO2e column</t>
-  </si>
-  <si>
-    <t>kg CO2e per kWh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generation factor used for Scope 2, as DESNZ advises - it covers emissions from producing the electricity the brand buys. </t>
-  </si>
-  <si>
-    <t>0 as REGO-backed renewable.</t>
-  </si>
-  <si>
-    <t>GHG Protocol Scope 2 Guidance (market-based method, Scope 2 Quality Criteria).</t>
-  </si>
-  <si>
-    <t>Coal</t>
-  </si>
-  <si>
-    <t>Natural Gas</t>
-  </si>
-  <si>
-    <t>Nuclear</t>
-  </si>
-  <si>
-    <t>Renewables</t>
-  </si>
-  <si>
-    <t>Other Fuels</t>
-  </si>
-  <si>
-    <t>Energy Source (%)</t>
-  </si>
-  <si>
-    <t>Intensity (g/kWh)</t>
-  </si>
-  <si>
-    <t>Weighted Average</t>
-  </si>
-  <si>
-    <t>Contribution (g/kWh)</t>
-  </si>
-  <si>
-    <t>Contribution (kg/kWh)</t>
-  </si>
-  <si>
-    <t>kg CO2 per kWh</t>
-  </si>
-  <si>
-    <t>Residual mix used because the landlord's tariff is unknown (emission factor hierarchy). In reality the brand would ask the landlord. Coal - 2024 intensity, since there was no coal generation in 2025</t>
-  </si>
-  <si>
-    <t>Calculated from DESNZ Fuel Mix Disclosure data table, residual fuel mix for April 2025 to March 2026, CO2 intensities for 2025</t>
+    <t>Energy Source</t>
   </si>
 </sst>
 </file>
@@ -379,11 +412,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color rgb="FF0000FF"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color rgb="FF0432FF"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -400,6 +428,11 @@
       <sz val="12"/>
       <name val="Aptos Narrow"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF0432FF"/>
+      <name val="Aptos Narrow"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -409,7 +442,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -417,20 +450,51 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -780,48 +844,50 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="B1" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B2" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="B4" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="B6" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -830,6 +896,100 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <cols>
+    <col min="1" max="1" width="15.1640625" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" customWidth="1"/>
+    <col min="3" max="3" width="21.33203125" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" s="8">
+        <f>SUMIFS(Calculations!J:J,Calculations!A:A, A2)</f>
+        <v>8.840041728000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="8">
+        <f>SUMIFS(Calculations!J:J, Calculations!A:A, A3, Calculations!B:B,B3)</f>
+        <v>4.2638061</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>94</v>
+      </c>
+      <c r="C4" s="18">
+        <f>SUMIFS(Calculations!J:J, Calculations!A:A, A4, Calculations!B:B,B4)</f>
+        <v>5.5556509645000016</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" s="9">
+        <f>C2+C3</f>
+        <v>13.103847828000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="9">
+        <f>C2+C4</f>
+        <v>14.395692692500003</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -838,10 +998,10 @@
     <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="70" customWidth="1"/>
+    <col min="5" max="5" width="70" style="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="17">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -854,45 +1014,45 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="17">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="19">
         <v>3</v>
       </c>
       <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="14" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:5">
+    <row r="3" spans="1:5" ht="17">
       <c r="A3" t="s">
         <v>5</v>
       </c>
       <c r="B3" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="19">
         <v>9</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" ht="17">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -906,67 +1066,67 @@
       <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" ht="17">
       <c r="A5" t="s">
         <v>13</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="19">
         <v>130</v>
       </c>
       <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="14" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" ht="34">
       <c r="A6" t="s">
         <v>13</v>
       </c>
       <c r="B6" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="19">
         <v>10</v>
       </c>
       <c r="D6" t="s">
         <v>18</v>
       </c>
-      <c r="E6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+      <c r="E6" s="14" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="17">
       <c r="A7" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2">
+        <v>19</v>
+      </c>
+      <c r="C7" s="19">
         <v>70</v>
       </c>
       <c r="D7" t="s">
         <v>15</v>
       </c>
-      <c r="E7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
+      <c r="E7" s="14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="17">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <f>C3*C6+C7</f>
@@ -975,238 +1135,202 @@
       <c r="D8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="34">
+      <c r="A9" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="9" spans="1:5">
-      <c r="A9" t="s">
+      <c r="B9" t="s">
         <v>24</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" s="19">
+        <v>108.01</v>
+      </c>
+      <c r="D9" t="s">
         <v>25</v>
       </c>
-      <c r="C9" s="2">
-        <v>108.01</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="E9" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="E9" t="s">
+    </row>
+    <row r="10" spans="1:5" ht="34">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" t="s">
+      <c r="C10" s="19">
+        <v>190.08</v>
+      </c>
+      <c r="D10" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="2">
-        <v>190.08</v>
-      </c>
-      <c r="D10" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" t="s">
+    </row>
+    <row r="11" spans="1:5" ht="68">
+      <c r="A11" t="s">
+        <v>23</v>
+      </c>
+      <c r="B11" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="11" spans="1:5">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" t="s">
+      <c r="C11" s="19">
+        <v>62.8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="E11" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="2">
-        <v>62.8</v>
-      </c>
-      <c r="D11" t="s">
-        <v>26</v>
-      </c>
-      <c r="E11" t="s">
+    </row>
+    <row r="12" spans="1:5" ht="34">
+      <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="12" spans="1:5">
-      <c r="A12" t="s">
-        <v>24</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="C12" s="19">
+        <v>147.54</v>
+      </c>
+      <c r="D12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="2">
-        <v>147.54</v>
-      </c>
-      <c r="D12" t="s">
-        <v>26</v>
-      </c>
-      <c r="E12" t="s">
+    </row>
+    <row r="13" spans="1:5" ht="17">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
         <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5">
-      <c r="A13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B13" t="s">
-        <v>34</v>
       </c>
       <c r="C13">
         <f>C5*C9</f>
         <v>14041.300000000001</v>
       </c>
       <c r="D13" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E13" t="s">
+    </row>
+    <row r="14" spans="1:5" ht="17">
+      <c r="A14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5">
-      <c r="A14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" t="s">
-        <v>37</v>
       </c>
       <c r="C14">
         <f>C5*C10</f>
         <v>24710.400000000001</v>
       </c>
       <c r="D14" t="s">
+        <v>34</v>
+      </c>
+      <c r="E14" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E14" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5">
+    </row>
+    <row r="15" spans="1:5" ht="17">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C15">
         <f>C8*C11</f>
         <v>10048</v>
       </c>
       <c r="D15" t="s">
+        <v>34</v>
+      </c>
+      <c r="E15" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5">
+    </row>
+    <row r="16" spans="1:5" ht="17">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C16">
         <f>C8*C12</f>
         <v>23606.399999999998</v>
       </c>
       <c r="D16" t="s">
+        <v>34</v>
+      </c>
+      <c r="E16" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="E16" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5">
+    </row>
+    <row r="17" spans="1:5" ht="34">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B17" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" t="s">
         <v>41</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="E17" t="s">
+    </row>
+    <row r="18" spans="1:5" ht="34">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="18" spans="1:5">
-      <c r="A18" t="s">
-        <v>24</v>
-      </c>
-      <c r="B18" t="s">
+      <c r="C18" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="D18" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="14" t="s">
         <v>45</v>
       </c>
-      <c r="D18" t="s">
-        <v>42</v>
-      </c>
-      <c r="E18" t="s">
-        <v>46</v>
-      </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" t="s">
-        <v>48</v>
-      </c>
       <c r="C19" s="2"/>
-      <c r="D19" t="s">
-        <v>49</v>
-      </c>
     </row>
     <row r="20" spans="1:5">
-      <c r="A20" t="s">
-        <v>47</v>
-      </c>
-      <c r="B20" t="s">
-        <v>50</v>
-      </c>
       <c r="C20" s="2"/>
-      <c r="D20" t="s">
-        <v>51</v>
-      </c>
     </row>
     <row r="21" spans="1:5">
-      <c r="A21" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21" t="s">
-        <v>52</v>
-      </c>
       <c r="C21" s="2"/>
-      <c r="D21" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="22" spans="1:5">
-      <c r="A22" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" t="s">
-        <v>54</v>
-      </c>
       <c r="C22" s="2"/>
-      <c r="D22" t="s">
-        <v>55</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
@@ -1216,123 +1340,123 @@
     <col min="3" max="3" width="10" customWidth="1"/>
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="7" width="50" customWidth="1"/>
+    <col min="6" max="7" width="50" style="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" ht="17">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="51">
+      <c r="A2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="19">
+        <v>0.18296000000000001</v>
+      </c>
+      <c r="D2" s="19" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
+      <c r="E2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F2" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="B2" t="s">
+      <c r="G2" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="C2" s="3">
-        <v>0.18296000000000001</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="E2" t="s">
+    </row>
+    <row r="3" spans="1:7" ht="51">
+      <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="19">
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F3" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="G3" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="3">
-        <v>0.17699999999999999</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E3" t="s">
-        <v>78</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+    </row>
+    <row r="4" spans="1:7" ht="68">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
-      </c>
-      <c r="C4" s="8">
+        <v>69</v>
+      </c>
+      <c r="C4" s="7">
         <f>'Residual mix'!E7</f>
         <v>0.39566500000000004</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>101</v>
+      <c r="D4" s="19" t="s">
+        <v>86</v>
       </c>
       <c r="E4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="34">
+      <c r="A5" t="s">
+        <v>70</v>
+      </c>
+      <c r="B5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="19">
+        <v>0</v>
+      </c>
+      <c r="D5" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5" t="s">
+        <v>67</v>
+      </c>
+      <c r="F5" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="20" t="s">
         <v>78</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="E5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>
@@ -1340,39 +1464,43 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87414153-6F28-2944-A156-CC2E49189BDE}">
   <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="15" style="4" customWidth="1"/>
+    <col min="1" max="1" width="15.1640625" customWidth="1"/>
+    <col min="2" max="2" width="15" style="3" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="17.6640625" customWidth="1"/>
     <col min="5" max="5" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
-      <c r="B1" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E1" t="s">
-        <v>100</v>
+      <c r="A1" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>91</v>
-      </c>
-      <c r="B2" s="5">
+        <v>80</v>
+      </c>
+      <c r="B2" s="4">
         <v>0.114</v>
       </c>
-      <c r="C2" s="6">
+      <c r="C2" s="5">
         <v>921</v>
       </c>
       <c r="D2">
@@ -1386,12 +1514,12 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B3" s="5">
+        <v>63</v>
+      </c>
+      <c r="B3" s="4">
         <v>0.65300000000000002</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="5">
         <v>365</v>
       </c>
       <c r="D3">
@@ -1405,12 +1533,12 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B4" s="5">
+        <v>81</v>
+      </c>
+      <c r="B4" s="4">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>0</v>
       </c>
       <c r="D4">
@@ -1424,12 +1552,12 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" t="s">
-        <v>94</v>
-      </c>
-      <c r="B5" s="5">
+        <v>82</v>
+      </c>
+      <c r="B5" s="4">
         <v>0.108</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="5">
         <v>0</v>
       </c>
       <c r="D5">
@@ -1443,12 +1571,12 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" t="s">
-        <v>95</v>
-      </c>
-      <c r="B6" s="5">
+        <v>110</v>
+      </c>
+      <c r="B6" s="4">
         <v>5.3999999999999999E-2</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="5">
         <v>969</v>
       </c>
       <c r="D6">
@@ -1462,7 +1590,7 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="D7">
         <f>SUM(D2:D6)</f>
@@ -1474,30 +1602,286 @@
       </c>
     </row>
     <row r="10" spans="1:5">
-      <c r="A10" s="7"/>
+      <c r="A10" s="6"/>
     </row>
     <row r="12" spans="1:5">
-      <c r="A12" s="7"/>
+      <c r="A12" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.33203125" customWidth="1"/>
+    <col min="2" max="2" width="14.1640625" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="12" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="23.33203125" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" style="8" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="E1" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="12">
+        <f>Assumptions!C14</f>
+        <v>24710.400000000001</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G2">
+        <f>_xlfn.XLOOKUP(F2, 'Emission factors'!A:A,'Emission factors'!C:C)</f>
+        <v>0.18296000000000001</v>
+      </c>
+      <c r="H2" t="str">
+        <f>_xlfn.XLOOKUP(F2,'Emission factors'!A:A,'Emission factors'!D:D)</f>
+        <v>kg CO2e per kWh (Gross CV)</v>
+      </c>
+      <c r="I2" s="8">
+        <f>E2*G2</f>
+        <v>4521.0147840000009</v>
+      </c>
+      <c r="J2" s="8">
+        <f>I2/1000</f>
+        <v>4.521014784000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E3" s="12">
+        <f>Assumptions!C16</f>
+        <v>23606.399999999998</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="G3">
+        <f>_xlfn.XLOOKUP(F3, 'Emission factors'!A:A,'Emission factors'!C:C)</f>
+        <v>0.18296000000000001</v>
+      </c>
+      <c r="H3" t="str">
+        <f>_xlfn.XLOOKUP(F3,'Emission factors'!A:A,'Emission factors'!D:D)</f>
+        <v>kg CO2e per kWh (Gross CV)</v>
+      </c>
+      <c r="I3" s="8">
+        <f t="shared" ref="I3:I7" si="0">E3*G3</f>
+        <v>4319.0269440000002</v>
+      </c>
+      <c r="J3" s="8">
+        <f t="shared" ref="J3:J7" si="1">I3/1000</f>
+        <v>4.319026944</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" t="s">
+        <v>98</v>
+      </c>
+      <c r="E4" s="12">
+        <f>Assumptions!C13</f>
+        <v>14041.300000000001</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G4">
+        <f>_xlfn.XLOOKUP(F4, 'Emission factors'!A:A,'Emission factors'!C:C)</f>
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="H4" t="str">
+        <f>_xlfn.XLOOKUP(F4,'Emission factors'!A:A,'Emission factors'!D:D)</f>
+        <v>kg CO2e per kWh</v>
+      </c>
+      <c r="I4" s="8">
+        <f t="shared" si="0"/>
+        <v>2485.3101000000001</v>
+      </c>
+      <c r="J4" s="8">
+        <f t="shared" si="1"/>
+        <v>2.4853101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D5" t="s">
+        <v>98</v>
+      </c>
+      <c r="E5" s="12">
+        <f>Assumptions!C15</f>
+        <v>10048</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="G5">
+        <f>_xlfn.XLOOKUP(F5, 'Emission factors'!A:A,'Emission factors'!C:C)</f>
+        <v>0.17699999999999999</v>
+      </c>
+      <c r="H5" t="str">
+        <f>_xlfn.XLOOKUP(F5,'Emission factors'!A:A,'Emission factors'!D:D)</f>
+        <v>kg CO2e per kWh</v>
+      </c>
+      <c r="I5" s="8">
+        <f t="shared" si="0"/>
+        <v>1778.4959999999999</v>
+      </c>
+      <c r="J5" s="8">
+        <f t="shared" si="1"/>
+        <v>1.7784959999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E6" s="12">
+        <f>Assumptions!C13</f>
+        <v>14041.300000000001</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6">
+        <f>_xlfn.XLOOKUP(F6, 'Emission factors'!A:A,'Emission factors'!C:C)</f>
+        <v>0.39566500000000004</v>
+      </c>
+      <c r="H6" t="str">
+        <f>_xlfn.XLOOKUP(F6,'Emission factors'!A:A,'Emission factors'!D:D)</f>
+        <v>kg CO2 per kWh</v>
+      </c>
+      <c r="I6" s="8">
+        <f t="shared" si="0"/>
+        <v>5555.6509645000015</v>
+      </c>
+      <c r="J6" s="8">
+        <f t="shared" si="1"/>
+        <v>5.5556509645000016</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D7" t="s">
+        <v>98</v>
+      </c>
+      <c r="E7" s="12">
+        <f>Assumptions!C15</f>
+        <v>10048</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7">
+        <f>_xlfn.XLOOKUP(F7, 'Emission factors'!A:A,'Emission factors'!C:C)</f>
+        <v>0</v>
+      </c>
+      <c r="H7" t="str">
+        <f>_xlfn.XLOOKUP(F7,'Emission factors'!A:A,'Emission factors'!D:D)</f>
+        <v>kg CO2e per kWh</v>
+      </c>
+      <c r="I7" s="8">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="8">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>